<commit_message>
Add RL_SM_01~09 safety mechanisms to both Excel files
- RL_SM_01: voltage protection only (no safe state activation)
- Add full braking/steering SM table with diagnostic coverage
- Add 安全机制 sheet to comparison checklist file

Co-authored-by: 杨玉辉 <13937083596@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/C255-10_SW_DFA报告.xlsx
+++ b/C255-10_SW_DFA报告.xlsx
@@ -423,7 +423,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$¥-804]#,##0.0000000000000;[$¥-804]\-#,##0.0000000000000"/>
   </numFmts>
-  <fonts count="81">
+  <fonts count="82">
     <font>
       <name val="Arial"/>
       <charset val="134"/>
@@ -963,8 +963,12 @@
       <color rgb="FF000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="52">
+  <fills count="53">
     <fill>
       <patternFill/>
     </fill>
@@ -1269,6 +1273,11 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -1871,7 +1880,7 @@
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="70" fillId="51" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="193">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="56">
       <alignment vertical="center"/>
@@ -2399,6 +2408,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="52" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="52" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="60">
@@ -6851,7 +6875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A2:Z27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.91666666666667" defaultRowHeight="14.5"/>
   <cols>
     <col width="17.3333333333333" customWidth="1" style="96" min="1" max="1"/>
@@ -6863,7 +6887,6 @@
     <col width="9.91666666666667" customWidth="1" style="98" min="43" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="54.5" customFormat="1" customHeight="1" s="93">
       <c r="A2" s="99" t="n"/>
       <c r="B2" s="99" t="n"/>
@@ -10276,7 +10299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="B1:O148"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.0833333333333" defaultRowHeight="15"/>
   <cols>
     <col width="3.33333333333333" customWidth="1" style="72" min="1" max="1"/>
@@ -13376,7 +13399,6 @@
       <c r="L1" s="159" t="n"/>
       <c r="M1" s="182" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="75" customFormat="1" customHeight="1" s="36">
       <c r="A3" s="30">
         <f>'[25]Top Event'!B4</f>
@@ -15158,7 +15180,6 @@
       <c r="H54" s="64" t="n"/>
       <c r="I54" s="64" t="n"/>
     </row>
-    <row r="55"/>
     <row r="56" ht="75" customFormat="1" customHeight="1" s="36">
       <c r="A56" s="67">
         <f>'[25]Top Event'!B5</f>
@@ -50958,123 +50979,385 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333333333333" defaultRowHeight="14" outlineLevelRow="6"/>
   <cols>
-    <col width="35.9166666666667" customWidth="1" min="1" max="1"/>
-    <col width="43.0833333333333" customWidth="1" min="2" max="2"/>
-    <col width="45.9166666666667" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>SM No.</t>
-        </is>
-      </c>
-      <c r="B1" s="13" t="inlineStr">
-        <is>
-          <t>Safety Mechanism Description</t>
-        </is>
-      </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="A1" s="188" t="inlineStr">
+        <is>
+          <t>功能</t>
+        </is>
+      </c>
+      <c r="B1" s="188" t="inlineStr">
+        <is>
+          <t>SM ID</t>
+        </is>
+      </c>
+      <c r="C1" s="188" t="inlineStr">
+        <is>
+          <t>安全机制</t>
+        </is>
+      </c>
+      <c r="D1" s="189" t="inlineStr">
         <is>
           <t>Traceability</t>
         </is>
       </c>
+      <c r="E1" s="189" t="inlineStr">
+        <is>
+          <t>诊断覆盖率</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="51" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_DFA_SM_001:
-</t>
-        </is>
-      </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="A2" s="190" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="B2" s="190" t="inlineStr">
+        <is>
+          <t>RL_SM_01</t>
+        </is>
+      </c>
+      <c r="C2" s="190" t="inlineStr">
+        <is>
+          <t>电源监控器检测违反稳定电源的错误，以确保整个系统的供电，包括过压和欠压保护。此SM负责处理和诊断电源问题。</t>
+        </is>
+      </c>
+      <c r="D2" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E2" s="191" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="43" customHeight="1">
+      <c r="A3" s="185" t="n"/>
+      <c r="B3" s="190" t="inlineStr">
+        <is>
+          <t>RL_SM_02</t>
+        </is>
+      </c>
+      <c r="C3" s="190" t="inlineStr">
+        <is>
+          <t>对来电信号进行检测，判断转向灯、制动灯是否满足开启要求；当来电信号错误，功能灯不响应，转向灯、制动灯各自进入安全状态（转向反馈、制动由车身检查）。</t>
+        </is>
+      </c>
+      <c r="D3" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E3" s="191" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="185" t="n"/>
+      <c r="B4" s="190" t="inlineStr">
+        <is>
+          <t>RL_SM_03</t>
+        </is>
+      </c>
+      <c r="C4" s="192" t="inlineStr">
+        <is>
+          <t>软件使用外部独立看门狗，当MCU软件故障可通过看门狗进行复位。</t>
+        </is>
+      </c>
+      <c r="D4" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E4" s="191" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
+      <c r="A5" s="185" t="n"/>
+      <c r="B5" s="190" t="inlineStr">
+        <is>
+          <t>RL_SM_04</t>
+        </is>
+      </c>
+      <c r="C5" s="192" t="inlineStr">
+        <is>
+          <t>灯具内部做故障判断逻辑，当判断故障后进行反馈，反馈机制应遵循奇瑞标准。</t>
+        </is>
+      </c>
+      <c r="D5" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E5" s="191" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="185" t="n"/>
+      <c r="B6" s="190" t="inlineStr">
+        <is>
+          <t>RL_SM_05</t>
+        </is>
+      </c>
+      <c r="C6" s="192" t="inlineStr">
+        <is>
+          <t>当制动灯内部故障且故障无法反馈时，由车身进行电流检测以此判断制动灯故障状态。</t>
+        </is>
+      </c>
+      <c r="D6" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E6" s="191" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="185" t="n"/>
+      <c r="B7" s="192" t="inlineStr">
+        <is>
+          <t>RL_SM_06</t>
+        </is>
+      </c>
+      <c r="C7" s="192" t="inlineStr">
+        <is>
+          <t>制动灯采用N-1&gt;=1方案进行设计，当某一组LED驱动或LED故障，剩余制动灯可以继续点亮。</t>
+        </is>
+      </c>
+      <c r="D7" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E7" s="191" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="185" t="n"/>
+      <c r="B8" s="191" t="inlineStr">
+        <is>
+          <t>RL_SM_07</t>
+        </is>
+      </c>
+      <c r="C8" s="191" t="inlineStr">
+        <is>
+          <t>转向灯采用N-1=0方案进行设计，当某一组LED驱动或LED故障，剩余转向灯熄灭。</t>
+        </is>
+      </c>
+      <c r="D8" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E8" s="191" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="185" t="n"/>
+      <c r="B9" s="191" t="inlineStr">
+        <is>
+          <t>RL_SM_08</t>
+        </is>
+      </c>
+      <c r="C9" s="191" t="inlineStr">
+        <is>
+          <t>在检测电路设计时，应考虑检测输出电压是否会导致MCU故障，故应使用钳位二极管将电压抑制在稳定区间。</t>
+        </is>
+      </c>
+      <c r="D9" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E9" s="191" t="inlineStr">
+        <is>
+          <t>99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="186" t="n"/>
+      <c r="B10" s="191" t="inlineStr">
+        <is>
+          <t>RL_SM_09</t>
+        </is>
+      </c>
+      <c r="C10" s="191" t="inlineStr">
+        <is>
+          <t>芯片硬件支持自检，并利用芯片特性设计外围电路。</t>
+        </is>
+      </c>
+      <c r="D10" s="191" t="inlineStr">
+        <is>
+          <t>制动转向</t>
+        </is>
+      </c>
+      <c r="E10" s="191" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SW DFA (软件)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>以下为 SW DFA 分析中引用的软件安全机制</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="191" t="inlineStr">
+        <is>
+          <t>SW_DFA_SM_001</t>
+        </is>
+      </c>
+      <c r="C13" s="191" t="inlineStr">
         <is>
           <t>支持硬线制动灯点亮</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="D13" s="191" t="inlineStr">
         <is>
           <t>SG1-硬线制动灯冗余</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="43" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_DFA_SM_002: </t>
-        </is>
-      </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="E13" s="191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="191" t="inlineStr">
+        <is>
+          <t>SW_DFA_SM_002</t>
+        </is>
+      </c>
+      <c r="C14" s="191" t="inlineStr">
         <is>
           <t>支持停振检测</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="D14" s="191" t="inlineStr">
         <is>
           <t>SG1/SG2/SG3-时钟停振检测</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_DFA_SM_003: </t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="E14" s="191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="191" t="inlineStr">
+        <is>
+          <t>SW_DFA_SM_003</t>
+        </is>
+      </c>
+      <c r="C15" s="191" t="inlineStr">
         <is>
           <t>制动灯报文丢失200ms后点亮制动灯</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="D15" s="191" t="inlineStr">
         <is>
           <t>SG1-报文丢失200ms制动灯点亮</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="39" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_DFA_SM_004: </t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="E15" s="191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="191" t="inlineStr">
+        <is>
+          <t>SW_DFA_SM_004</t>
+        </is>
+      </c>
+      <c r="C16" s="191" t="inlineStr">
         <is>
           <t>支持外部看门狗</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="D16" s="191" t="inlineStr">
         <is>
           <t>SG1/SG2/SG3-外部看门狗</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SW_DFA_SM_005: </t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="E16" s="191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="191" t="inlineStr">
+        <is>
+          <t>SW_DFA_SM_005</t>
+        </is>
+      </c>
+      <c r="C17" s="191" t="inlineStr">
         <is>
           <t>连续10个周期BCC校验失败后会点亮制动灯</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="D17" s="191" t="inlineStr">
         <is>
           <t>SG1-BCC校验失败制动灯点亮</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="18" t="n"/>
-      <c r="C7" s="19" t="n"/>
+      <c r="E17" s="191" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:A10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>